<commit_message>
Excel file changed to meet new format specs.
  Changes to be committed:
	modified:   TestLab Network Configuration Details.xlsx
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E44C255D-CC24-4122-B864-5C330044B544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86917DC5-0596-4B6C-8C2D-B765EE88CCDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Network Ovierview &amp; DHCP" sheetId="2" r:id="rId1"/>
+    <sheet name="Node Details" sheetId="3" r:id="rId2"/>
+    <sheet name="IP &amp; DNS Configuration" sheetId="4" r:id="rId3"/>
+    <sheet name="Original Data to be Moved" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -971,6 +974,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6525761-94DF-4000-BA36-A56D05134533}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A018CAD-CC25-408D-B297-7CA78622B82C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A499D3-5D72-450B-A081-DFA6BEAA292C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21CAD797-1037-4B44-A397-368C91E19BD7}">
   <dimension ref="B1:I21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add content to network configuration XLSX file...
  Changes to the excel file:
  * Added the network overview section to the Network Overview & DHCP sheet
  * Moved the old DHCP Organization Table to the Overview & DHCP sheet
  * Created 2 tables on the Node Details sheet, one for permanent nodes
	and one for temporary and/or testing nodes
  * Data for the Node Details sheet will be entered later
  * Moved the old IP Assignments table to the new DNS & IP sheet
  * Since the Old Data sheet was now empty, it was deleted
  * Created a better font/color theme that was deployed to some of the
	sheets - it will be deployed to all sheets in the next Excel commit

  Changes to be committed:
    modified:   TestLab Network Configuration Details.xlsx
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86917DC5-0596-4B6C-8C2D-B765EE88CCDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01E84DC-E4D5-4714-83B6-8001892BA02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43260" yWindow="2070" windowWidth="28770" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4065" yWindow="2670" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Network Ovierview &amp; DHCP" sheetId="2" r:id="rId1"/>
     <sheet name="Node Details" sheetId="3" r:id="rId2"/>
-    <sheet name="IP &amp; DNS Configuration" sheetId="4" r:id="rId3"/>
-    <sheet name="Original Data to be Moved" sheetId="1" r:id="rId4"/>
+    <sheet name="Lab DNS &amp; IP Assignments" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="87">
   <si>
     <t>Testlab Network:</t>
   </si>
@@ -201,13 +200,109 @@
   </si>
   <si>
     <t># of Hosts in IP Range</t>
+  </si>
+  <si>
+    <t>Node's DNS Name</t>
+  </si>
+  <si>
+    <t>Node's Focal Points or Purpose</t>
+  </si>
+  <si>
+    <t>Node's Operating System</t>
+  </si>
+  <si>
+    <t>Testing and/or Temporary Nodes</t>
+  </si>
+  <si>
+    <t>Permanent Nodes</t>
+  </si>
+  <si>
+    <t>(Physical/Virtual)</t>
+  </si>
+  <si>
+    <t>Node's Purpose and/or Focal Points</t>
+  </si>
+  <si>
+    <t>Test Lab Network Node Descriptions</t>
+  </si>
+  <si>
+    <t>Network Overview</t>
+  </si>
+  <si>
+    <t>Network Overview &amp;</t>
+  </si>
+  <si>
+    <t>DHCP Scope Configuration</t>
+  </si>
+  <si>
+    <t>Network Feature</t>
+  </si>
+  <si>
+    <t>DHCP Scope Organization</t>
+  </si>
+  <si>
+    <t>on the Test Lab's Primary Subnet</t>
+  </si>
+  <si>
+    <t>Lab's Primary Subnet:</t>
+  </si>
+  <si>
+    <t>Varible's Value</t>
+  </si>
+  <si>
+    <t>Relevent Notes</t>
+  </si>
+  <si>
+    <t>IP Version</t>
+  </si>
+  <si>
+    <t>Main Lab Subnets</t>
+  </si>
+  <si>
+    <t>Network Address Bits</t>
+  </si>
+  <si>
+    <t># of Nodes/Subnet</t>
+  </si>
+  <si>
+    <t>Auxiliary Subnets</t>
+  </si>
+  <si>
+    <t>For testing only…</t>
+  </si>
+  <si>
+    <t>(Including 4-Port Gateway)</t>
+  </si>
+  <si>
+    <t>Switch Ports/Subnet</t>
+  </si>
+  <si>
+    <t>Switchs/Subnet</t>
+  </si>
+  <si>
+    <t>POE Ports/Subnet</t>
+  </si>
+  <si>
+    <t>Subnet Speed</t>
+  </si>
+  <si>
+    <t>1Gb</t>
+  </si>
+  <si>
+    <t>Bonded Connections</t>
+  </si>
+  <si>
+    <t>Main Nodes/Servers</t>
+  </si>
+  <si>
+    <t>Bonded from 2 1Gb Links</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,15 +346,63 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FF7A0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <i/>
       <sz val="12"/>
-      <color rgb="FF00B050"/>
+      <color rgb="FF7030A0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="6" tint="-0.24994659260841701"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color theme="9" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -353,16 +496,6 @@
     <fill>
       <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
         <stop position="0">
-          <color theme="7" tint="0.80001220740379042"/>
-        </stop>
-        <stop position="1">
-          <color theme="8" tint="0.80001220740379042"/>
-        </stop>
-      </gradientFill>
-    </fill>
-    <fill>
-      <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
-        <stop position="0">
           <color theme="4" tint="0.80001220740379042"/>
         </stop>
         <stop position="1">
@@ -370,8 +503,26 @@
         </stop>
       </gradientFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -581,19 +732,231 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color auto="1"/>
+      </left>
+      <right style="double">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="double">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="double">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="double">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -604,9 +967,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
@@ -626,14 +987,80 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="15" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="15" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="15" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="16" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="16" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="16" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="16" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="16" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="10" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="10" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -642,6 +1069,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF7A0000"/>
       <color rgb="FFFF3F3F"/>
       <color rgb="FFFF6161"/>
       <color rgb="FFFF9393"/>
@@ -975,373 +1403,733 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6525761-94DF-4000-BA36-A56D05134533}">
-  <dimension ref="A1"/>
+  <dimension ref="C1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" customWidth="1"/>
+    <col min="9" max="9" width="61.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="42" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="44" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="3:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="H5" s="44" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="48" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="48" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="47" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="64" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="65">
+        <v>4</v>
+      </c>
+      <c r="E7" s="66"/>
+      <c r="G7" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="64" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="65">
+        <v>1</v>
+      </c>
+      <c r="E8" s="66"/>
+      <c r="G8" s="52">
+        <v>1</v>
+      </c>
+      <c r="H8" s="56" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="67" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="65">
+        <v>24</v>
+      </c>
+      <c r="E9" s="66"/>
+      <c r="G9" s="53">
+        <v>18</v>
+      </c>
+      <c r="H9" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="64" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="65">
+        <v>254</v>
+      </c>
+      <c r="E10" s="66"/>
+      <c r="G10" s="53">
+        <v>69</v>
+      </c>
+      <c r="H10" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="63" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="65">
+        <v>3</v>
+      </c>
+      <c r="E11" s="66" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="53">
+        <v>8</v>
+      </c>
+      <c r="H11" s="59" t="s">
+        <v>19</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="65">
+        <v>46</v>
+      </c>
+      <c r="E12" s="66"/>
+      <c r="G12" s="53">
+        <v>19</v>
+      </c>
+      <c r="H12" s="60" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="65">
+        <v>18</v>
+      </c>
+      <c r="E13" s="66"/>
+      <c r="G13" s="53">
+        <v>120</v>
+      </c>
+      <c r="H13" s="61" t="s">
+        <v>51</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="66"/>
+      <c r="G14" s="54">
+        <v>13</v>
+      </c>
+      <c r="H14" s="62" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="3:9" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="65" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="66" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="55">
+        <f>SUM(G8:G14)</f>
+        <v>248</v>
+      </c>
+      <c r="H15" s="33" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="64" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="65">
+        <v>1</v>
+      </c>
+      <c r="E16" s="66" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A018CAD-CC25-408D-B297-7CA78622B82C}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:E37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="43.5703125" customWidth="1"/>
+    <col min="5" max="5" width="115.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D2" s="41" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="37" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="39"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="39"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="39"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="39"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="39"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+    </row>
+    <row r="19" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="40"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+    </row>
+    <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="37" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="39"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="39"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="39"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="39"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="39"/>
+      <c r="E31" s="39"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="39"/>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="39"/>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="39"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="39"/>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="39"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="39"/>
+    </row>
+    <row r="36" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="40"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="40"/>
+    </row>
+    <row r="37" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A499D3-5D72-450B-A081-DFA6BEAA292C}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:E22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="28.85546875" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="17">
+        <v>1</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="20">
+        <v>1</v>
+      </c>
+      <c r="E7" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="23">
+        <v>1</v>
+      </c>
+      <c r="E8" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="23">
+        <v>2</v>
+      </c>
+      <c r="E9" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="26">
+        <v>0</v>
+      </c>
+      <c r="E10" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="26">
+        <v>0</v>
+      </c>
+      <c r="E11" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="26">
+        <v>0</v>
+      </c>
+      <c r="E12" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="26">
+        <v>0</v>
+      </c>
+      <c r="E13" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="26">
+        <v>0</v>
+      </c>
+      <c r="E14" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="26">
+        <v>0</v>
+      </c>
+      <c r="E15" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="26">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0</v>
+      </c>
+      <c r="E17" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0</v>
+      </c>
+      <c r="E18" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="11">
+        <v>1</v>
+      </c>
+      <c r="E19" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="6">
+        <f>SUM(D6:D18)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="2">
+        <f>SUM(E6:E20)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21CAD797-1037-4B44-A397-368C91E19BD7}">
-  <dimension ref="B1:I21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" customWidth="1"/>
-    <col min="8" max="8" width="26.42578125" customWidth="1"/>
-    <col min="9" max="9" width="60.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="37" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H2" s="40" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="40" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="39" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="36" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4">
-        <v>18</v>
-      </c>
-      <c r="H4" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="23">
-        <v>1</v>
-      </c>
-      <c r="E5" s="24">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>69</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="26">
-        <v>1</v>
-      </c>
-      <c r="E6" s="27">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="19" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="29">
-        <v>1</v>
-      </c>
-      <c r="E7" s="30">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>19</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="29">
-        <v>2</v>
-      </c>
-      <c r="E8" s="30">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>120</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="32">
-        <v>0</v>
-      </c>
-      <c r="E9" s="33">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>13</v>
-      </c>
-      <c r="H9" s="41" t="s">
-        <v>52</v>
-      </c>
-      <c r="I9" s="17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="32">
-        <v>0</v>
-      </c>
-      <c r="E10" s="33">
-        <v>0</v>
-      </c>
-      <c r="G10" s="42">
-        <f>SUM(G3:G9)</f>
-        <v>248</v>
-      </c>
-      <c r="H10" s="43" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="32">
-        <v>0</v>
-      </c>
-      <c r="E11" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="32">
-        <v>0</v>
-      </c>
-      <c r="E12" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="32">
-        <v>0</v>
-      </c>
-      <c r="E13" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="32">
-        <v>0</v>
-      </c>
-      <c r="E14" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="32">
-        <v>0</v>
-      </c>
-      <c r="E15" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="12">
-        <v>0</v>
-      </c>
-      <c r="E16" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="12">
-        <v>0</v>
-      </c>
-      <c r="E17" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="15">
-        <v>1</v>
-      </c>
-      <c r="E18" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="10">
-        <f>SUM(D5:D17)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D20" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="2">
-        <f>SUM(E5:E19)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add DHCP Reservation Config to Services Section
  * Added the Pi Hole DHCP IP 4 Address Reservation Details to the Services Section
  * Fixed a Minor Error in the Lab Configuration XLSX file

  Changes to be committed:
    new file:   Services/PI Hole DHCP IP 4 Address Reservation List.md
	modified:   TestLab Network Configuration Details.xlsx
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01E84DC-E4D5-4714-83B6-8001892BA02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6FFB2B-E521-4B47-8C14-CF5E8B9D203A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4065" yWindow="2670" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38805" yWindow="3060" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Network Ovierview &amp; DHCP" sheetId="2" r:id="rId1"/>
     <sheet name="Node Details" sheetId="3" r:id="rId2"/>
     <sheet name="Lab DNS &amp; IP Assignments" sheetId="4" r:id="rId3"/>
+    <sheet name="Core Network Services" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="93">
   <si>
     <t>Testlab Network:</t>
   </si>
@@ -296,6 +297,24 @@
   </si>
   <si>
     <t>Bonded from 2 1Gb Links</t>
+  </si>
+  <si>
+    <t>10.0.2.240</t>
+  </si>
+  <si>
+    <t>Core Network Services</t>
+  </si>
+  <si>
+    <t>Provided by Node</t>
+  </si>
+  <si>
+    <t>Provided on Port #</t>
+  </si>
+  <si>
+    <t>Network Service</t>
+  </si>
+  <si>
+    <t>NebulonW-SVVM</t>
   </si>
 </sst>
 </file>
@@ -1047,14 +1066,14 @@
     <xf numFmtId="1" fontId="10" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="10" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1874,7 +1893,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A499D3-5D72-450B-A081-DFA6BEAA292C}">
-  <dimension ref="B2:E22"/>
+  <dimension ref="B2:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.28515625" customWidth="1"/>
@@ -2069,25 +2088,25 @@
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="8">
+      <c r="B17" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="26">
         <v>0</v>
       </c>
-      <c r="E17" s="9">
-        <v>1</v>
+      <c r="E17" s="27">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D18" s="8">
         <v>0</v>
@@ -2096,39 +2115,87 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="10" t="s">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="8">
+        <v>0</v>
+      </c>
+      <c r="E19" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C20" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D20" s="11">
         <v>1</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E20" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="5" t="s">
+    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="6">
-        <f>SUM(D6:D18)</f>
+      <c r="D21" s="6">
+        <f>SUM(D6:D19)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D21" s="1" t="s">
+    <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="2">
-        <f>SUM(E6:E20)</f>
+      <c r="E22" s="2">
+        <f>SUM(E6:E21)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428EB2F2-668A-4E29-B34A-1506874D8B93}">
+  <dimension ref="B1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D2" s="41" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update DNS/DHCP Assignment Table on the XLSX Doc
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6FFB2B-E521-4B47-8C14-CF5E8B9D203A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E9C670-7478-42D9-9AD1-5EC71AD916A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38805" yWindow="3060" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -182,12 +182,6 @@
     <t>10.0.2.182</t>
   </si>
   <si>
-    <t>10.0.2.183</t>
-  </si>
-  <si>
-    <t>Hole-RPSV PiHole (DNS Srv)</t>
-  </si>
-  <si>
     <t>10.0.2.21 - 10.0.2.90</t>
   </si>
   <si>
@@ -315,6 +309,12 @@
   </si>
   <si>
     <t>NebulonW-SVVM</t>
+  </si>
+  <si>
+    <t>10.0.2.156</t>
+  </si>
+  <si>
+    <t>RPI-Hole-SV</t>
   </si>
 </sst>
 </file>
@@ -1442,37 +1442,37 @@
         <v>2</v>
       </c>
       <c r="D2" s="43" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="3:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D5" s="46" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H5" s="44" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="48" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H6" s="47" t="s">
         <v>1</v>
@@ -1480,14 +1480,14 @@
     </row>
     <row r="7" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="64" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D7" s="65">
         <v>4</v>
       </c>
       <c r="E7" s="66"/>
       <c r="G7" s="51" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H7" s="50" t="s">
         <v>18</v>
@@ -1498,7 +1498,7 @@
     </row>
     <row r="8" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="64" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D8" s="65">
         <v>1</v>
@@ -1516,7 +1516,7 @@
     </row>
     <row r="9" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="67" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D9" s="65">
         <v>24</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="10" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="64" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D10" s="65">
         <v>254</v>
@@ -1544,7 +1544,7 @@
         <v>69</v>
       </c>
       <c r="H10" s="58" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I10" s="63" t="s">
         <v>24</v>
@@ -1552,13 +1552,13 @@
     </row>
     <row r="11" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="64" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D11" s="65">
         <v>3</v>
       </c>
       <c r="E11" s="66" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G11" s="53">
         <v>8</v>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="12" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="64" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D12" s="65">
         <v>46</v>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="13" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="64" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D13" s="65">
         <v>18</v>
@@ -1600,7 +1600,7 @@
         <v>120</v>
       </c>
       <c r="H13" s="61" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>27</v>
@@ -1608,17 +1608,17 @@
     </row>
     <row r="14" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="64" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D14" s="65" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E14" s="66"/>
       <c r="G14" s="54">
         <v>13</v>
       </c>
       <c r="H14" s="62" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I14" s="13" t="s">
         <v>26</v>
@@ -1626,31 +1626,31 @@
     </row>
     <row r="15" spans="3:9" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="66" t="s">
         <v>84</v>
-      </c>
-      <c r="D15" s="65" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>86</v>
       </c>
       <c r="G15" s="55">
         <f>SUM(G8:G14)</f>
         <v>248</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="64" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D16" s="65">
         <v>1</v>
       </c>
       <c r="E16" s="66" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -1674,27 +1674,27 @@
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D4" s="37" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="34" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C5" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="D5" s="35" t="s">
-        <v>57</v>
-      </c>
       <c r="E5" s="36" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -1784,21 +1784,21 @@
     <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D21" s="37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="34" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C22" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="35" t="s">
-        <v>57</v>
-      </c>
       <c r="E22" s="36" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -2019,10 +2019,10 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D12" s="26">
         <v>0</v>
@@ -2033,10 +2033,10 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="D13" s="26">
         <v>0</v>
@@ -2047,10 +2047,10 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D14" s="26">
         <v>0</v>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="25" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D15" s="26">
         <v>0</v>
@@ -2075,10 +2075,10 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="25" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" s="26">
         <v>0</v>
@@ -2089,10 +2089,10 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D17" s="26">
         <v>0</v>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="20" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="10" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>34</v>
@@ -2164,6 +2164,7 @@
     <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2181,19 +2182,19 @@
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="41" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Details of the TL-OSINT-WSVM Node to XLSX.
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E9C670-7478-42D9-9AD1-5EC71AD916A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D32C0-5416-4DB7-A15F-4D8DD0F3D630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38805" yWindow="3060" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="95">
   <si>
     <t>Testlab Network:</t>
   </si>
@@ -164,9 +164,6 @@
     <t>10.0.2.180</t>
   </si>
   <si>
-    <t>tlosint-WSVM</t>
-  </si>
-  <si>
     <t>10.0.2.181</t>
   </si>
   <si>
@@ -315,6 +312,15 @@
   </si>
   <si>
     <t>RPI-Hole-SV</t>
+  </si>
+  <si>
+    <t>NebulonR-SVVM</t>
+  </si>
+  <si>
+    <t>10.0.2.183</t>
+  </si>
+  <si>
+    <t>tl-osint-WSVM</t>
   </si>
 </sst>
 </file>
@@ -1442,37 +1448,37 @@
         <v>2</v>
       </c>
       <c r="D2" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="44" t="s">
         <v>62</v>
-      </c>
-      <c r="E2" s="44" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="3:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="3:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D5" s="46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G5" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="44" t="s">
         <v>65</v>
-      </c>
-      <c r="H5" s="44" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D6" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="48" t="s">
-        <v>69</v>
-      </c>
       <c r="G6" s="45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H6" s="47" t="s">
         <v>1</v>
@@ -1480,14 +1486,14 @@
     </row>
     <row r="7" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="64" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D7" s="65">
         <v>4</v>
       </c>
       <c r="E7" s="66"/>
       <c r="G7" s="51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H7" s="50" t="s">
         <v>18</v>
@@ -1498,7 +1504,7 @@
     </row>
     <row r="8" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="64" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D8" s="65">
         <v>1</v>
@@ -1516,7 +1522,7 @@
     </row>
     <row r="9" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="67" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="65">
         <v>24</v>
@@ -1534,7 +1540,7 @@
     </row>
     <row r="10" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="64" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" s="65">
         <v>254</v>
@@ -1544,7 +1550,7 @@
         <v>69</v>
       </c>
       <c r="H10" s="58" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I10" s="63" t="s">
         <v>24</v>
@@ -1552,13 +1558,13 @@
     </row>
     <row r="11" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="64" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="65">
         <v>3</v>
       </c>
       <c r="E11" s="66" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G11" s="53">
         <v>8</v>
@@ -1572,7 +1578,7 @@
     </row>
     <row r="12" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="64" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="65">
         <v>46</v>
@@ -1590,7 +1596,7 @@
     </row>
     <row r="13" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="64" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D13" s="65">
         <v>18</v>
@@ -1600,7 +1606,7 @@
         <v>120</v>
       </c>
       <c r="H13" s="61" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>27</v>
@@ -1608,17 +1614,17 @@
     </row>
     <row r="14" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="65" t="s">
         <v>80</v>
-      </c>
-      <c r="D14" s="65" t="s">
-        <v>81</v>
       </c>
       <c r="E14" s="66"/>
       <c r="G14" s="54">
         <v>13</v>
       </c>
       <c r="H14" s="62" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I14" s="13" t="s">
         <v>26</v>
@@ -1626,31 +1632,31 @@
     </row>
     <row r="15" spans="3:9" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="65" t="s">
+      <c r="E15" s="66" t="s">
         <v>83</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>84</v>
       </c>
       <c r="G15" s="55">
         <f>SUM(G8:G14)</f>
         <v>248</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="3:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D16" s="65">
         <v>1</v>
       </c>
       <c r="E16" s="66" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -1674,27 +1680,27 @@
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D4" s="37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="36" t="s">
         <v>53</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="E5" s="36" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -1784,21 +1790,21 @@
     <row r="20" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D21" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="36" t="s">
         <v>58</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="D22" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="36" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -1893,7 +1899,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A499D3-5D72-450B-A081-DFA6BEAA292C}">
-  <dimension ref="B2:E23"/>
+  <dimension ref="B2:E24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.28515625" customWidth="1"/>
@@ -1991,10 +1997,10 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="26" t="s">
         <v>44</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>45</v>
       </c>
       <c r="D10" s="26">
         <v>0</v>
@@ -2022,7 +2028,7 @@
         <v>37</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D12" s="26">
         <v>0</v>
@@ -2061,10 +2067,10 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="26" t="s">
         <v>42</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>43</v>
       </c>
       <c r="D15" s="26">
         <v>0</v>
@@ -2075,10 +2081,10 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="26" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>47</v>
       </c>
       <c r="D16" s="26">
         <v>0</v>
@@ -2089,10 +2095,10 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="25" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D17" s="26">
         <v>0</v>
@@ -2102,25 +2108,25 @@
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="8">
+      <c r="B18" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="26">
         <v>0</v>
       </c>
-      <c r="E18" s="9">
-        <v>1</v>
+      <c r="E18" s="27">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D19" s="8">
         <v>0</v>
@@ -2129,39 +2135,53 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="11" t="s">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="8">
+        <v>0</v>
+      </c>
+      <c r="E20" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D21" s="11">
         <v>1</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E21" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="5" t="s">
+    <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="6">
-        <f>SUM(D6:D19)</f>
+      <c r="D22" s="6">
+        <f>SUM(D6:D20)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D22" s="1" t="s">
+    <row r="23" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E22" s="2">
-        <f>SUM(E6:E21)</f>
+      <c r="E23" s="2">
+        <f>SUM(E6:E22)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2182,19 +2202,19 @@
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" s="41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" t="s">
         <v>87</v>
-      </c>
-      <c r="E4" t="s">
-        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clarify and Unify XLSX Table Design Across Sheets
</commit_message>
<xml_diff>
--- a/TestLab Network Configuration Details.xlsx
+++ b/TestLab Network Configuration Details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FSO\Homeone-TestLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D32C0-5416-4DB7-A15F-4D8DD0F3D630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BAC1FD2-AE48-4B5F-B479-6A6989EED61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38805" yWindow="3060" windowWidth="28770" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38805" yWindow="3060" windowWidth="28770" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Network Ovierview &amp; DHCP" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="104">
   <si>
     <t>Testlab Network:</t>
   </si>
@@ -321,13 +321,40 @@
   </si>
   <si>
     <t>tl-osint-WSVM</t>
+  </si>
+  <si>
+    <t>KradFish-WSVM</t>
+  </si>
+  <si>
+    <t>10.0.2.170</t>
+  </si>
+  <si>
+    <t>Homeone Test Lab's</t>
+  </si>
+  <si>
+    <t>DNS</t>
+  </si>
+  <si>
+    <t>DHCP</t>
+  </si>
+  <si>
+    <t>Proxmox Web App</t>
+  </si>
+  <si>
+    <t>Service Types:</t>
+  </si>
+  <si>
+    <t>Locally Hosted Service</t>
+  </si>
+  <si>
+    <t>Cloud Hosted Service</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,8 +453,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="8" tint="-0.24994659260841701"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -546,8 +581,20 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="35">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -973,11 +1020,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1086,6 +1163,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1529,7 +1622,7 @@
       </c>
       <c r="E9" s="66"/>
       <c r="G9" s="53">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H9" s="57" t="s">
         <v>20</v>
@@ -1547,7 +1640,7 @@
       </c>
       <c r="E10" s="66"/>
       <c r="G10" s="53">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H10" s="58" t="s">
         <v>47</v>
@@ -1567,7 +1660,7 @@
         <v>75</v>
       </c>
       <c r="G11" s="53">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11" s="59" t="s">
         <v>19</v>
@@ -1585,7 +1678,7 @@
       </c>
       <c r="E12" s="66"/>
       <c r="G12" s="53">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H12" s="60" t="s">
         <v>21</v>
@@ -1603,7 +1696,7 @@
       </c>
       <c r="E13" s="66"/>
       <c r="G13" s="53">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H13" s="61" t="s">
         <v>48</v>
@@ -1621,7 +1714,7 @@
       </c>
       <c r="E14" s="66"/>
       <c r="G14" s="54">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H14" s="62" t="s">
         <v>49</v>
@@ -1642,7 +1735,7 @@
       </c>
       <c r="G15" s="55">
         <f>SUM(G8:G14)</f>
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="H15" s="33" t="s">
         <v>50</v>
@@ -1899,7 +1992,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A499D3-5D72-450B-A081-DFA6BEAA292C}">
-  <dimension ref="B2:E24"/>
+  <dimension ref="B2:E25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.28515625" customWidth="1"/>
@@ -2053,10 +2146,10 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>41</v>
+        <v>96</v>
       </c>
       <c r="D14" s="26">
         <v>0</v>
@@ -2067,10 +2160,10 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="25" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D15" s="26">
         <v>0</v>
@@ -2081,10 +2174,10 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="25" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D16" s="26">
         <v>0</v>
@@ -2095,10 +2188,10 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="25" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="D17" s="26">
         <v>0</v>
@@ -2109,10 +2202,10 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="25" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="D18" s="26">
         <v>0</v>
@@ -2122,25 +2215,25 @@
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="8">
+      <c r="B19" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="26">
         <v>0</v>
       </c>
-      <c r="E19" s="9">
-        <v>1</v>
+      <c r="E19" s="27">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D20" s="8">
         <v>0</v>
@@ -2149,39 +2242,53 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="10" t="s">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0</v>
+      </c>
+      <c r="E21" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C22" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D22" s="11">
         <v>1</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E22" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="5" t="s">
+    <row r="23" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="6">
-        <f>SUM(D6:D20)</f>
+      <c r="D23" s="6">
+        <f>SUM(D6:D21)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D23" s="1" t="s">
+    <row r="24" spans="2:5" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="2">
-        <f>SUM(E6:E22)</f>
+      <c r="E24" s="2">
+        <f>SUM(E6:E23)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2190,34 +2297,230 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428EB2F2-668A-4E29-B34A-1506874D8B93}">
-  <dimension ref="B1:E4"/>
+  <dimension ref="B1:G32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="29.140625" customWidth="1"/>
     <col min="4" max="4" width="27" customWidth="1"/>
     <col min="5" max="5" width="18.85546875" customWidth="1"/>
+    <col min="7" max="7" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:5" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D2" s="41" t="s">
+    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="68" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="68" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+    <row r="3" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C3" s="69"/>
+      <c r="D3" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E3" s="69" t="s">
         <v>87</v>
       </c>
+    </row>
+    <row r="4" spans="2:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="71" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="71"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="71" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="71"/>
+      <c r="D6" s="71"/>
+      <c r="E6" s="71"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="71"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="71"/>
+      <c r="E7" s="71"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="71"/>
+      <c r="C8" s="71"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="71"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="71"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="71"/>
+      <c r="C10" s="71"/>
+      <c r="D10" s="71"/>
+      <c r="E10" s="71"/>
+    </row>
+    <row r="11" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="71"/>
+      <c r="C11" s="71"/>
+      <c r="D11" s="71"/>
+      <c r="E11" s="71"/>
+    </row>
+    <row r="12" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="71"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="71"/>
+      <c r="E12" s="71"/>
+      <c r="G12" s="72" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="71"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="71"/>
+      <c r="E13" s="71"/>
+      <c r="G13" s="73" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+      <c r="G14" s="74" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="71"/>
+      <c r="C15" s="71"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="71"/>
+      <c r="G15" s="75"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="71"/>
+      <c r="C16" s="71"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="71"/>
+      <c r="G16" s="75"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="71"/>
+      <c r="C17" s="71"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="71"/>
+      <c r="C18" s="71"/>
+      <c r="D18" s="71"/>
+      <c r="E18" s="71"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="71"/>
+      <c r="C19" s="71"/>
+      <c r="D19" s="71"/>
+      <c r="E19" s="71"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="71"/>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="71"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="71"/>
+      <c r="C22" s="71"/>
+      <c r="D22" s="71"/>
+      <c r="E22" s="71"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="71"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="71"/>
+      <c r="E23" s="71"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="70"/>
+      <c r="C24" s="70"/>
+      <c r="D24" s="70"/>
+      <c r="E24" s="70"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="70"/>
+      <c r="C25" s="70"/>
+      <c r="D25" s="70"/>
+      <c r="E25" s="70"/>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="70"/>
+      <c r="C26" s="70"/>
+      <c r="D26" s="70"/>
+      <c r="E26" s="70"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="70"/>
+      <c r="C27" s="70"/>
+      <c r="D27" s="70"/>
+      <c r="E27" s="70"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="70"/>
+      <c r="C28" s="70"/>
+      <c r="D28" s="70"/>
+      <c r="E28" s="70"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="70"/>
+      <c r="C29" s="70"/>
+      <c r="D29" s="70"/>
+      <c r="E29" s="70"/>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="70"/>
+      <c r="C30" s="70"/>
+      <c r="D30" s="70"/>
+      <c r="E30" s="70"/>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="70"/>
+      <c r="C31" s="70"/>
+      <c r="D31" s="70"/>
+      <c r="E31" s="70"/>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="70"/>
+      <c r="C32" s="70"/>
+      <c r="D32" s="70"/>
+      <c r="E32" s="70"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>